<commit_message>
excel updates Conteúdo e layout de página para site | Site Layouts para stand eventos patrocinados | Layout para stand Eventos patrocinados: KV | KV de eventos KV - Contempla conteúdo e layout | KV de mobilização
</commit_message>
<xml_diff>
--- a/runrun_report/Escopo Nuclea.xlsx
+++ b/runrun_report/Escopo Nuclea.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caiofs\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9583B48B-997D-4953-B233-DE9ABB930893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7ED2E4-3A2D-4852-8184-947E65D9CB77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2250" yWindow="2310" windowWidth="18900" windowHeight="10965" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9300" yWindow="3000" windowWidth="12540" windowHeight="10965" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="79">
   <si>
     <t>PROJETO</t>
   </si>
@@ -192,9 +192,6 @@
     <t>E-mails de convite eventos patrocinados</t>
   </si>
   <si>
-    <t>Layouts para stand eventos patrocinados</t>
-  </si>
-  <si>
     <t>E-mails de convite Núclea Day</t>
   </si>
   <si>
@@ -261,29 +258,29 @@
     <t>Site</t>
   </si>
   <si>
-    <t>Conteúdo e layout de página para site</t>
-  </si>
-  <si>
     <t>Eventos</t>
   </si>
   <si>
-    <t xml:space="preserve">Eventos Patrocinados: KV </t>
-  </si>
-  <si>
-    <t>KV - Contempla conteúdo e layout</t>
-  </si>
-  <si>
     <t>Peças gráficas de mobilização</t>
   </si>
   <si>
     <t>Peças gráficas de eventos</t>
+  </si>
+  <si>
+    <t>Layout para stand</t>
+  </si>
+  <si>
+    <t>KV de eventos</t>
+  </si>
+  <si>
+    <t>KV de mobilização</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -328,14 +325,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -701,7 +690,7 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1462,24 +1451,24 @@
   <sheetData>
     <row r="2" spans="2:6">
       <c r="B2" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="25" t="s">
         <v>67</v>
-      </c>
-      <c r="C2" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="F2" s="25" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>41</v>
@@ -1497,13 +1486,13 @@
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4" s="26" t="s">
         <v>42</v>
       </c>
       <c r="D4" s="27">
-        <f t="shared" ref="D4:D31" si="0">E4/12</f>
+        <f t="shared" ref="D4:D29" si="0">E4/12</f>
         <v>12</v>
       </c>
       <c r="E4" s="27">
@@ -1515,7 +1504,7 @@
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5" s="26" t="s">
         <v>43</v>
@@ -1533,7 +1522,7 @@
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C6" s="26" t="s">
         <v>44</v>
@@ -1551,7 +1540,7 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C7" s="26" t="s">
         <v>45</v>
@@ -1602,7 +1591,7 @@
     </row>
     <row r="10" spans="2:6">
       <c r="B10" s="26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C10" s="26" t="s">
         <v>47</v>
@@ -1620,10 +1609,10 @@
     </row>
     <row r="11" spans="2:6">
       <c r="B11" s="28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D11" s="27"/>
       <c r="E11" s="29">
@@ -1635,7 +1624,7 @@
     </row>
     <row r="12" spans="2:6">
       <c r="B12" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C12" s="32" t="s">
         <v>50</v>
@@ -1650,7 +1639,7 @@
     </row>
     <row r="13" spans="2:6">
       <c r="B13" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C13" s="26" t="s">
         <v>48</v>
@@ -1665,7 +1654,7 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C14" s="26" t="s">
         <v>49</v>
@@ -1680,10 +1669,10 @@
     </row>
     <row r="15" spans="2:6">
       <c r="B15" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="28" t="s">
         <v>75</v>
-      </c>
-      <c r="C15" s="28" t="s">
-        <v>79</v>
       </c>
       <c r="D15" s="27"/>
       <c r="E15" s="29">
@@ -1695,10 +1684,10 @@
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="35" t="s">
-        <v>51</v>
+        <v>73</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>76</v>
       </c>
       <c r="D16" s="27"/>
       <c r="E16" s="27">
@@ -1710,10 +1699,10 @@
     </row>
     <row r="17" spans="2:6">
       <c r="B17" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D17" s="27"/>
       <c r="E17" s="27">
@@ -1725,10 +1714,10 @@
     </row>
     <row r="18" spans="2:6">
       <c r="B18" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D18" s="27">
         <f t="shared" si="0"/>
@@ -1743,10 +1732,10 @@
     </row>
     <row r="19" spans="2:6">
       <c r="B19" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D19" s="27">
         <f t="shared" si="0"/>
@@ -1761,10 +1750,10 @@
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="27">
         <f t="shared" si="0"/>
@@ -1779,10 +1768,10 @@
     </row>
     <row r="21" spans="2:6">
       <c r="B21" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="27">
         <f t="shared" si="0"/>
@@ -1797,10 +1786,10 @@
     </row>
     <row r="22" spans="2:6">
       <c r="B22" s="26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="27"/>
       <c r="E22" s="27">
@@ -1815,7 +1804,7 @@
         <v>29</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="27">
         <f t="shared" si="0"/>
@@ -1833,7 +1822,7 @@
         <v>29</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D24" s="27">
         <f t="shared" si="0"/>
@@ -1850,8 +1839,8 @@
       <c r="B25" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="30" t="s">
-        <v>77</v>
+      <c r="C25" s="35" t="s">
+        <v>78</v>
       </c>
       <c r="D25" s="27"/>
       <c r="E25" s="31">
@@ -1866,7 +1855,7 @@
         <v>29</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D26" s="27">
         <f t="shared" si="0"/>
@@ -1884,7 +1873,7 @@
         <v>29</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D27" s="27">
         <f t="shared" si="0"/>
@@ -1902,7 +1891,7 @@
         <v>29</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D28" s="27">
         <f t="shared" si="0"/>
@@ -1920,7 +1909,7 @@
         <v>29</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D29" s="27">
         <f t="shared" si="0"/>
@@ -1938,7 +1927,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D30" s="27"/>
       <c r="E30" s="34">
@@ -1953,7 +1942,7 @@
         <v>29</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D31" s="27"/>
       <c r="E31" s="34">

</xml_diff>